<commit_message>
feat(s24-t1): parseWhen + announce registration (TABS/FPRINT/GID/template/fingerprints; D5 13→14)
</commit_message>
<xml_diff>
--- a/tools/gfy-template.xlsx
+++ b/tools/gfy-template.xlsx
@@ -20,6 +20,7 @@
     <sheet name="Shame" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Invites" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Rooms" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Announce" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1011,6 +1012,67 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>when</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-08-14 18:05</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SAMPLE — Draft complete. See the Draft tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-08-16 07:40</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SAMPLE — R2 tee times posted. Leaders out last.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>